<commit_message>
* Improved `test_run_one_year.py` to create a spreadsheet  output to verify calculations ... see file `test_run_one_year_DATE_with_formulas.xlsx` for the formulas * Fine-tuned `run_montecarlo_simulation.py`
###
</commit_message>
<xml_diff>
--- a/Data/Morningstar_asset_stats_2025_12_21.xlsx
+++ b/Data/Morningstar_asset_stats_2025_12_21.xlsx
@@ -1,10 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="4" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="124226"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bfraenkel/Documents/Code/Financial_Plan/Data/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{85FBF581-6E0E-7A41-99FB-278A42174B18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660"/>
+    <workbookView xWindow="15500" yWindow="1300" windowWidth="13140" windowHeight="18960" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Stats" sheetId="1" r:id="rId1"/>
@@ -15,7 +21,20 @@
     <sheet name="Model" sheetId="6" r:id="rId6"/>
     <sheet name="Stock-Bond Ratios" sheetId="7" r:id="rId7"/>
   </sheets>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -484,8 +503,8 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -537,10 +556,33 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -548,13 +590,21 @@
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme 2007 - 2010">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2007 - 2010">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -592,7 +642,7 @@
         <a:srgbClr val="800080"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2007 - 2010">
       <a:majorFont>
         <a:latin typeface="Cambria"/>
         <a:ea typeface=""/>
@@ -626,6 +676,7 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Times New Roman"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -660,9 +711,10 @@
         <a:font script="Mong" typeface="Mongolian Baiti"/>
         <a:font script="Viet" typeface="Arial"/>
         <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2007 - 2010">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -835,26 +887,30 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:D15"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="27.1640625" style="4" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:4">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:4" s="3" customFormat="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="6" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" s="5" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="5" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="2" spans="1:4">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" s="7" t="s">
         <v>4</v>
       </c>
       <c r="B2">
@@ -867,8 +923,8 @@
         <v>1.91</v>
       </c>
     </row>
-    <row r="3" spans="1:4">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" s="7" t="s">
         <v>5</v>
       </c>
       <c r="B3">
@@ -881,8 +937,8 @@
         <v>2.8</v>
       </c>
     </row>
-    <row r="4" spans="1:4">
-      <c r="A4" s="1" t="s">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="7" t="s">
         <v>6</v>
       </c>
       <c r="B4">
@@ -892,25 +948,25 @@
         <v>21.65</v>
       </c>
       <c r="D4">
-        <v>1.15</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4">
-      <c r="A5" s="1" t="s">
+        <v>1.1499999999999999</v>
+      </c>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="7" t="s">
         <v>7</v>
       </c>
       <c r="B5">
         <v>10.09</v>
       </c>
       <c r="C5">
-        <v>16.6</v>
+        <v>16.600000000000001</v>
       </c>
       <c r="D5">
         <v>2.48</v>
       </c>
     </row>
-    <row r="6" spans="1:4">
-      <c r="A6" s="1" t="s">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" s="7" t="s">
         <v>8</v>
       </c>
       <c r="B6">
@@ -923,22 +979,22 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="7" spans="1:4">
-      <c r="A7" s="1" t="s">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" s="7" t="s">
         <v>9</v>
       </c>
       <c r="B7">
         <v>10.86</v>
       </c>
       <c r="C7">
-        <v>18.9</v>
+        <v>18.899999999999999</v>
       </c>
       <c r="D7">
         <v>2.19</v>
       </c>
     </row>
-    <row r="8" spans="1:4">
-      <c r="A8" s="1" t="s">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B8">
@@ -951,8 +1007,8 @@
         <v>3.27</v>
       </c>
     </row>
-    <row r="9" spans="1:4">
-      <c r="A9" s="1" t="s">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" s="7" t="s">
         <v>11</v>
       </c>
       <c r="B9">
@@ -965,8 +1021,8 @@
         <v>2.78</v>
       </c>
     </row>
-    <row r="10" spans="1:4">
-      <c r="A10" s="1" t="s">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" s="7" t="s">
         <v>12</v>
       </c>
       <c r="B10">
@@ -979,22 +1035,22 @@
         <v>4.05</v>
       </c>
     </row>
-    <row r="11" spans="1:4">
-      <c r="A11" s="1" t="s">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" s="7" t="s">
         <v>13</v>
       </c>
       <c r="B11">
         <v>6.58</v>
       </c>
       <c r="C11">
-        <v>9.609999999999999</v>
+        <v>9.61</v>
       </c>
       <c r="D11">
         <v>9.48</v>
       </c>
     </row>
-    <row r="12" spans="1:4">
-      <c r="A12" s="1" t="s">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" s="7" t="s">
         <v>14</v>
       </c>
       <c r="B12">
@@ -1007,8 +1063,8 @@
         <v>2.73</v>
       </c>
     </row>
-    <row r="13" spans="1:4">
-      <c r="A13" s="1" t="s">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" s="7" t="s">
         <v>15</v>
       </c>
       <c r="B13">
@@ -1021,8 +1077,8 @@
         <v>2.04</v>
       </c>
     </row>
-    <row r="14" spans="1:4">
-      <c r="A14" s="1" t="s">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" s="7" t="s">
         <v>16</v>
       </c>
       <c r="B14">
@@ -1035,8 +1091,8 @@
         <v>2.04</v>
       </c>
     </row>
-    <row r="15" spans="1:4">
-      <c r="A15" s="1" t="s">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" s="7" t="s">
         <v>17</v>
       </c>
       <c r="B15">
@@ -1055,712 +1111,716 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:O15"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="27.1640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="15" width="10.83203125" style="9" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="1" spans="1:15">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:15" ht="47" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A1" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="8" t="s">
         <v>5</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="8" t="s">
         <v>7</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="8" t="s">
         <v>8</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="8" t="s">
         <v>11</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" s="8" t="s">
         <v>15</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" s="8" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:15">
-      <c r="A2" s="1" t="s">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A2" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="B2">
+      <c r="B2" s="10">
         <v>1</v>
       </c>
-      <c r="C2">
+      <c r="C2" s="10">
         <v>0.85</v>
       </c>
-      <c r="D2">
+      <c r="D2" s="10">
         <v>0.9</v>
       </c>
-      <c r="E2">
+      <c r="E2" s="10">
         <v>0.74</v>
       </c>
-      <c r="F2">
+      <c r="F2" s="10">
         <v>0.86</v>
       </c>
-      <c r="G2">
+      <c r="G2" s="10">
         <v>0.72</v>
       </c>
-      <c r="H2">
-        <v>0.58</v>
-      </c>
-      <c r="I2">
+      <c r="H2" s="10">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="I2" s="10">
         <v>0.52</v>
       </c>
-      <c r="J2">
+      <c r="J2" s="10">
         <v>0.19</v>
       </c>
-      <c r="K2">
+      <c r="K2" s="10">
         <v>0.53</v>
       </c>
-      <c r="L2">
-        <v>0.01</v>
-      </c>
-      <c r="M2">
-        <v>0.02</v>
-      </c>
-      <c r="N2">
+      <c r="L2" s="10">
+        <v>0.01</v>
+      </c>
+      <c r="M2" s="10">
+        <v>0.02</v>
+      </c>
+      <c r="N2" s="10">
         <v>0.12</v>
       </c>
-      <c r="O2">
+      <c r="O2" s="10">
         <v>0.44</v>
       </c>
     </row>
-    <row r="3" spans="1:15">
-      <c r="A3" s="1" t="s">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="B3">
+      <c r="B3" s="10">
         <v>0.85</v>
       </c>
-      <c r="C3">
+      <c r="C3" s="10">
         <v>1</v>
       </c>
-      <c r="D3">
+      <c r="D3" s="10">
         <v>0.78</v>
       </c>
-      <c r="E3">
+      <c r="E3" s="10">
         <v>0.9</v>
       </c>
-      <c r="F3">
+      <c r="F3" s="10">
         <v>0.74</v>
       </c>
-      <c r="G3">
+      <c r="G3" s="10">
         <v>0.84</v>
       </c>
-      <c r="H3">
+      <c r="H3" s="10">
         <v>0.59</v>
       </c>
-      <c r="I3">
+      <c r="I3" s="10">
         <v>0.54</v>
       </c>
-      <c r="J3">
+      <c r="J3" s="10">
         <v>0.23</v>
       </c>
-      <c r="K3">
-        <v>0.58</v>
-      </c>
-      <c r="L3">
+      <c r="K3" s="10">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="L3" s="10">
         <v>-0.01</v>
       </c>
-      <c r="M3">
+      <c r="M3" s="10">
         <v>0.05</v>
       </c>
-      <c r="N3">
-        <v>0.14</v>
-      </c>
-      <c r="O3">
+      <c r="N3" s="10">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="O3" s="10">
         <v>0.59</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
-      <c r="A4" s="1" t="s">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A4" s="2" t="s">
         <v>6</v>
       </c>
-      <c r="B4">
+      <c r="B4" s="10">
         <v>0.9</v>
       </c>
-      <c r="C4">
+      <c r="C4" s="10">
         <v>0.78</v>
       </c>
-      <c r="D4">
+      <c r="D4" s="10">
         <v>1</v>
       </c>
-      <c r="E4">
+      <c r="E4" s="10">
         <v>0.78</v>
       </c>
-      <c r="F4">
+      <c r="F4" s="10">
         <v>0.98</v>
       </c>
-      <c r="G4">
+      <c r="G4" s="10">
         <v>0.79</v>
       </c>
-      <c r="H4">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="I4">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="J4">
+      <c r="H4" s="10">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="I4" s="10">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="J4" s="10">
         <v>0.12</v>
       </c>
-      <c r="K4">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="L4">
+      <c r="K4" s="10">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="L4" s="10">
         <v>-0.02</v>
       </c>
-      <c r="M4">
+      <c r="M4" s="10">
         <v>-0.02</v>
       </c>
-      <c r="N4">
+      <c r="N4" s="10">
         <v>0.16</v>
       </c>
-      <c r="O4">
+      <c r="O4" s="10">
         <v>0.52</v>
       </c>
     </row>
-    <row r="5" spans="1:15">
-      <c r="A5" s="1" t="s">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A5" s="2" t="s">
         <v>7</v>
       </c>
-      <c r="B5">
+      <c r="B5" s="10">
         <v>0.74</v>
       </c>
-      <c r="C5">
+      <c r="C5" s="10">
         <v>0.9</v>
       </c>
-      <c r="D5">
+      <c r="D5" s="10">
         <v>0.78</v>
       </c>
-      <c r="E5">
+      <c r="E5" s="10">
         <v>1</v>
       </c>
-      <c r="F5">
+      <c r="F5" s="10">
         <v>0.77</v>
       </c>
-      <c r="G5">
+      <c r="G5" s="10">
         <v>0.96</v>
       </c>
-      <c r="H5">
+      <c r="H5" s="10">
         <v>0.54</v>
       </c>
-      <c r="I5">
+      <c r="I5" s="10">
         <v>0.51</v>
       </c>
-      <c r="J5">
+      <c r="J5" s="10">
         <v>0.21</v>
       </c>
-      <c r="K5">
+      <c r="K5" s="10">
         <v>0.62</v>
       </c>
-      <c r="L5">
+      <c r="L5" s="10">
         <v>-0.01</v>
       </c>
-      <c r="M5">
-        <v>-0</v>
-      </c>
-      <c r="N5">
+      <c r="M5" s="10">
+        <v>0</v>
+      </c>
+      <c r="N5" s="10">
         <v>0.15</v>
       </c>
-      <c r="O5">
+      <c r="O5" s="10">
         <v>0.68</v>
       </c>
     </row>
-    <row r="6" spans="1:15">
-      <c r="A6" s="1" t="s">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A6" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B6">
+      <c r="B6" s="10">
         <v>0.86</v>
       </c>
-      <c r="C6">
+      <c r="C6" s="10">
         <v>0.74</v>
       </c>
-      <c r="D6">
+      <c r="D6" s="10">
         <v>0.98</v>
       </c>
-      <c r="E6">
+      <c r="E6" s="10">
         <v>0.77</v>
       </c>
-      <c r="F6">
+      <c r="F6" s="10">
         <v>1</v>
       </c>
-      <c r="G6">
-        <v>0.8100000000000001</v>
-      </c>
-      <c r="H6">
+      <c r="G6" s="10">
+        <v>0.81</v>
+      </c>
+      <c r="H6" s="10">
         <v>0.54</v>
       </c>
-      <c r="I6">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="J6">
+      <c r="I6" s="10">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="J6" s="10">
         <v>0.1</v>
       </c>
-      <c r="K6">
-        <v>0.58</v>
-      </c>
-      <c r="L6">
+      <c r="K6" s="10">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="L6" s="10">
         <v>-0.04</v>
       </c>
-      <c r="M6">
+      <c r="M6" s="10">
         <v>-0.04</v>
       </c>
-      <c r="N6">
+      <c r="N6" s="10">
         <v>0.16</v>
       </c>
-      <c r="O6">
+      <c r="O6" s="10">
         <v>0.54</v>
       </c>
     </row>
-    <row r="7" spans="1:15">
-      <c r="A7" s="1" t="s">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A7" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B7">
+      <c r="B7" s="10">
         <v>0.72</v>
       </c>
-      <c r="C7">
+      <c r="C7" s="10">
         <v>0.84</v>
       </c>
-      <c r="D7">
+      <c r="D7" s="10">
         <v>0.79</v>
       </c>
-      <c r="E7">
+      <c r="E7" s="10">
         <v>0.96</v>
       </c>
-      <c r="F7">
-        <v>0.8100000000000001</v>
-      </c>
-      <c r="G7">
+      <c r="F7" s="10">
+        <v>0.81</v>
+      </c>
+      <c r="G7" s="10">
         <v>1</v>
       </c>
-      <c r="H7">
+      <c r="H7" s="10">
         <v>0.52</v>
       </c>
-      <c r="I7">
+      <c r="I7" s="10">
         <v>0.52</v>
       </c>
-      <c r="J7">
+      <c r="J7" s="10">
         <v>0.16</v>
       </c>
-      <c r="K7">
+      <c r="K7" s="10">
         <v>0.64</v>
       </c>
-      <c r="L7">
+      <c r="L7" s="10">
         <v>-0.03</v>
       </c>
-      <c r="M7">
+      <c r="M7" s="10">
         <v>-0.01</v>
       </c>
-      <c r="N7">
+      <c r="N7" s="10">
         <v>0.16</v>
       </c>
-      <c r="O7">
+      <c r="O7" s="10">
         <v>0.7</v>
       </c>
     </row>
-    <row r="8" spans="1:15">
-      <c r="A8" s="1" t="s">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A8" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B8">
-        <v>0.58</v>
-      </c>
-      <c r="C8">
+      <c r="B8" s="10">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="C8" s="10">
         <v>0.59</v>
       </c>
-      <c r="D8">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="E8">
+      <c r="D8" s="10">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="E8" s="10">
         <v>0.54</v>
       </c>
-      <c r="F8">
+      <c r="F8" s="10">
         <v>0.54</v>
       </c>
-      <c r="G8">
+      <c r="G8" s="10">
         <v>0.52</v>
       </c>
-      <c r="H8">
+      <c r="H8" s="10">
         <v>1</v>
       </c>
-      <c r="I8">
+      <c r="I8" s="10">
         <v>0.67</v>
       </c>
-      <c r="J8">
+      <c r="J8" s="10">
         <v>0.17</v>
       </c>
-      <c r="K8">
+      <c r="K8" s="10">
         <v>0.4</v>
       </c>
-      <c r="L8">
-        <v>0.29</v>
-      </c>
-      <c r="M8">
+      <c r="L8" s="10">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="M8" s="10">
         <v>0.05</v>
       </c>
-      <c r="N8">
+      <c r="N8" s="10">
         <v>0.18</v>
       </c>
-      <c r="O8">
+      <c r="O8" s="10">
         <v>0.39</v>
       </c>
     </row>
-    <row r="9" spans="1:15">
-      <c r="A9" s="1" t="s">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A9" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="B9">
+      <c r="B9" s="10">
         <v>0.52</v>
       </c>
-      <c r="C9">
+      <c r="C9" s="10">
         <v>0.54</v>
       </c>
-      <c r="D9">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="E9">
+      <c r="D9" s="10">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="E9" s="10">
         <v>0.51</v>
       </c>
-      <c r="F9">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="G9">
+      <c r="F9" s="10">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="G9" s="10">
         <v>0.52</v>
       </c>
-      <c r="H9">
+      <c r="H9" s="10">
         <v>0.67</v>
       </c>
-      <c r="I9">
+      <c r="I9" s="10">
         <v>1</v>
       </c>
-      <c r="J9">
+      <c r="J9" s="10">
         <v>0.04</v>
       </c>
-      <c r="K9">
+      <c r="K9" s="10">
         <v>0.43</v>
       </c>
-      <c r="L9">
+      <c r="L9" s="10">
         <v>0.03</v>
       </c>
-      <c r="M9">
-        <v>0</v>
-      </c>
-      <c r="N9">
+      <c r="M9" s="10">
+        <v>0</v>
+      </c>
+      <c r="N9" s="10">
         <v>0.2</v>
       </c>
-      <c r="O9">
+      <c r="O9" s="10">
         <v>0.34</v>
       </c>
     </row>
-    <row r="10" spans="1:15">
-      <c r="A10" s="1" t="s">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A10" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B10">
+      <c r="B10" s="10">
         <v>0.19</v>
       </c>
-      <c r="C10">
+      <c r="C10" s="10">
         <v>0.23</v>
       </c>
-      <c r="D10">
+      <c r="D10" s="10">
         <v>0.12</v>
       </c>
-      <c r="E10">
+      <c r="E10" s="10">
         <v>0.21</v>
       </c>
-      <c r="F10">
+      <c r="F10" s="10">
         <v>0.1</v>
       </c>
-      <c r="G10">
+      <c r="G10" s="10">
         <v>0.16</v>
       </c>
-      <c r="H10">
+      <c r="H10" s="10">
         <v>0.17</v>
       </c>
-      <c r="I10">
+      <c r="I10" s="10">
         <v>0.04</v>
       </c>
-      <c r="J10">
+      <c r="J10" s="10">
         <v>1</v>
       </c>
-      <c r="K10">
+      <c r="K10" s="10">
         <v>0.38</v>
       </c>
-      <c r="L10">
+      <c r="L10" s="10">
         <v>0.45</v>
       </c>
-      <c r="M10">
+      <c r="M10" s="10">
         <v>0.24</v>
       </c>
-      <c r="N10">
+      <c r="N10" s="10">
         <v>-0.11</v>
       </c>
-      <c r="O10">
+      <c r="O10" s="10">
         <v>0.16</v>
       </c>
     </row>
-    <row r="11" spans="1:15">
-      <c r="A11" s="1" t="s">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A11" s="2" t="s">
         <v>13</v>
       </c>
-      <c r="B11">
+      <c r="B11" s="10">
         <v>0.53</v>
       </c>
-      <c r="C11">
-        <v>0.58</v>
-      </c>
-      <c r="D11">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="E11">
+      <c r="C11" s="10">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="D11" s="10">
+        <v>0.56000000000000005</v>
+      </c>
+      <c r="E11" s="10">
         <v>0.62</v>
       </c>
-      <c r="F11">
-        <v>0.58</v>
-      </c>
-      <c r="G11">
+      <c r="F11" s="10">
+        <v>0.57999999999999996</v>
+      </c>
+      <c r="G11" s="10">
         <v>0.64</v>
       </c>
-      <c r="H11">
+      <c r="H11" s="10">
         <v>0.4</v>
       </c>
-      <c r="I11">
+      <c r="I11" s="10">
         <v>0.43</v>
       </c>
-      <c r="J11">
+      <c r="J11" s="10">
         <v>0.38</v>
       </c>
-      <c r="K11">
+      <c r="K11" s="10">
         <v>1</v>
       </c>
-      <c r="L11">
+      <c r="L11" s="10">
         <v>0.08</v>
       </c>
-      <c r="M11">
-        <v>0.01</v>
-      </c>
-      <c r="N11">
+      <c r="M11" s="10">
+        <v>0.01</v>
+      </c>
+      <c r="N11" s="10">
         <v>0.04</v>
       </c>
-      <c r="O11">
+      <c r="O11" s="10">
         <v>0.5</v>
       </c>
     </row>
-    <row r="12" spans="1:15">
-      <c r="A12" s="1" t="s">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A12" s="2" t="s">
         <v>14</v>
       </c>
-      <c r="B12">
-        <v>0.01</v>
-      </c>
-      <c r="C12">
+      <c r="B12" s="10">
+        <v>0.01</v>
+      </c>
+      <c r="C12" s="10">
         <v>-0.01</v>
       </c>
-      <c r="D12">
+      <c r="D12" s="10">
         <v>-0.02</v>
       </c>
-      <c r="E12">
+      <c r="E12" s="10">
         <v>-0.01</v>
       </c>
-      <c r="F12">
+      <c r="F12" s="10">
         <v>-0.04</v>
       </c>
-      <c r="G12">
+      <c r="G12" s="10">
         <v>-0.03</v>
       </c>
-      <c r="H12">
-        <v>0.29</v>
-      </c>
-      <c r="I12">
+      <c r="H12" s="10">
+        <v>0.28999999999999998</v>
+      </c>
+      <c r="I12" s="10">
         <v>0.03</v>
       </c>
-      <c r="J12">
+      <c r="J12" s="10">
         <v>0.45</v>
       </c>
-      <c r="K12">
+      <c r="K12" s="10">
         <v>0.08</v>
       </c>
-      <c r="L12">
+      <c r="L12" s="10">
         <v>1</v>
       </c>
-      <c r="M12">
+      <c r="M12" s="10">
         <v>0.23</v>
       </c>
-      <c r="N12">
+      <c r="N12" s="10">
         <v>-0.08</v>
       </c>
-      <c r="O12">
-        <v>-0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15">
-      <c r="A13" s="1" t="s">
+      <c r="O12" s="10">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A13" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="B13">
-        <v>0.02</v>
-      </c>
-      <c r="C13">
+      <c r="B13" s="10">
+        <v>0.02</v>
+      </c>
+      <c r="C13" s="10">
         <v>0.05</v>
       </c>
-      <c r="D13">
+      <c r="D13" s="10">
         <v>-0.02</v>
       </c>
-      <c r="E13">
-        <v>-0</v>
-      </c>
-      <c r="F13">
+      <c r="E13" s="10">
+        <v>0</v>
+      </c>
+      <c r="F13" s="10">
         <v>-0.04</v>
       </c>
-      <c r="G13">
+      <c r="G13" s="10">
         <v>-0.01</v>
       </c>
-      <c r="H13">
+      <c r="H13" s="10">
         <v>0.05</v>
       </c>
-      <c r="I13">
-        <v>0</v>
-      </c>
-      <c r="J13">
+      <c r="I13" s="10">
+        <v>0</v>
+      </c>
+      <c r="J13" s="10">
         <v>0.24</v>
       </c>
-      <c r="K13">
-        <v>0.01</v>
-      </c>
-      <c r="L13">
+      <c r="K13" s="10">
+        <v>0.01</v>
+      </c>
+      <c r="L13" s="10">
         <v>0.23</v>
       </c>
-      <c r="M13">
+      <c r="M13" s="10">
         <v>1</v>
       </c>
-      <c r="N13">
+      <c r="N13" s="10">
         <v>-0.16</v>
       </c>
-      <c r="O13">
+      <c r="O13" s="10">
         <v>-0.05</v>
       </c>
     </row>
-    <row r="14" spans="1:15">
-      <c r="A14" s="1" t="s">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A14" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="B14">
+      <c r="B14" s="10">
         <v>0.12</v>
       </c>
-      <c r="C14">
-        <v>0.14</v>
-      </c>
-      <c r="D14">
+      <c r="C14" s="10">
+        <v>0.14000000000000001</v>
+      </c>
+      <c r="D14" s="10">
         <v>0.16</v>
       </c>
-      <c r="E14">
+      <c r="E14" s="10">
         <v>0.15</v>
       </c>
-      <c r="F14">
+      <c r="F14" s="10">
         <v>0.16</v>
       </c>
-      <c r="G14">
+      <c r="G14" s="10">
         <v>0.16</v>
       </c>
-      <c r="H14">
+      <c r="H14" s="10">
         <v>0.18</v>
       </c>
-      <c r="I14">
+      <c r="I14" s="10">
         <v>0.2</v>
       </c>
-      <c r="J14">
+      <c r="J14" s="10">
         <v>-0.11</v>
       </c>
-      <c r="K14">
+      <c r="K14" s="10">
         <v>0.04</v>
       </c>
-      <c r="L14">
+      <c r="L14" s="10">
         <v>-0.08</v>
       </c>
-      <c r="M14">
+      <c r="M14" s="10">
         <v>-0.16</v>
       </c>
-      <c r="N14">
+      <c r="N14" s="10">
         <v>1</v>
       </c>
-      <c r="O14">
+      <c r="O14" s="10">
         <v>0.16</v>
       </c>
     </row>
-    <row r="15" spans="1:15">
-      <c r="A15" s="1" t="s">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
+      <c r="A15" s="2" t="s">
         <v>17</v>
       </c>
-      <c r="B15">
+      <c r="B15" s="10">
         <v>0.44</v>
       </c>
-      <c r="C15">
+      <c r="C15" s="10">
         <v>0.59</v>
       </c>
-      <c r="D15">
+      <c r="D15" s="10">
         <v>0.52</v>
       </c>
-      <c r="E15">
+      <c r="E15" s="10">
         <v>0.68</v>
       </c>
-      <c r="F15">
+      <c r="F15" s="10">
         <v>0.54</v>
       </c>
-      <c r="G15">
+      <c r="G15" s="10">
         <v>0.7</v>
       </c>
-      <c r="H15">
+      <c r="H15" s="10">
         <v>0.39</v>
       </c>
-      <c r="I15">
+      <c r="I15" s="10">
         <v>0.34</v>
       </c>
-      <c r="J15">
+      <c r="J15" s="10">
         <v>0.16</v>
       </c>
-      <c r="K15">
+      <c r="K15" s="10">
         <v>0.5</v>
       </c>
-      <c r="L15">
-        <v>-0</v>
-      </c>
-      <c r="M15">
+      <c r="L15" s="10">
+        <v>0</v>
+      </c>
+      <c r="M15" s="10">
         <v>-0.05</v>
       </c>
-      <c r="N15">
+      <c r="N15" s="10">
         <v>0.16</v>
       </c>
-      <c r="O15">
+      <c r="O15" s="10">
         <v>1</v>
       </c>
     </row>
@@ -1770,11 +1830,11 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:O15"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B1" s="1" t="s">
         <v>4</v>
       </c>
@@ -1818,7 +1878,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:15">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -1841,7 +1901,7 @@
         <v>0.72</v>
       </c>
       <c r="H2">
-        <v>0.58</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="I2">
         <v>0.52</v>
@@ -1865,7 +1925,7 @@
         <v>0.44</v>
       </c>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -1897,7 +1957,7 @@
         <v>0.23</v>
       </c>
       <c r="K3">
-        <v>0.58</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="L3">
         <v>-0.01</v>
@@ -1906,13 +1966,13 @@
         <v>0.05</v>
       </c>
       <c r="N3">
-        <v>0.14</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="O3">
         <v>0.59</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -1935,16 +1995,16 @@
         <v>0.79</v>
       </c>
       <c r="H4">
-        <v>0.5600000000000001</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="I4">
-        <v>0.5600000000000001</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="J4">
         <v>0.12</v>
       </c>
       <c r="K4">
-        <v>0.5600000000000001</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="L4">
         <v>-0.02</v>
@@ -1959,7 +2019,7 @@
         <v>0.51</v>
       </c>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
@@ -1997,7 +2057,7 @@
         <v>-0.01</v>
       </c>
       <c r="M5">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="N5">
         <v>0.15</v>
@@ -2006,7 +2066,7 @@
         <v>0.68</v>
       </c>
     </row>
-    <row r="6" spans="1:15">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
@@ -2032,13 +2092,13 @@
         <v>0.54</v>
       </c>
       <c r="I6">
-        <v>0.5600000000000001</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="J6">
         <v>0.1</v>
       </c>
       <c r="K6">
-        <v>0.58</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="L6">
         <v>-0.04</v>
@@ -2053,7 +2113,7 @@
         <v>0.54</v>
       </c>
     </row>
-    <row r="7" spans="1:15">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
@@ -2100,18 +2160,18 @@
         <v>0.7</v>
       </c>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B8">
-        <v>0.58</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="C8">
         <v>0.59</v>
       </c>
       <c r="D8">
-        <v>0.5600000000000001</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="E8">
         <v>0.54</v>
@@ -2135,7 +2195,7 @@
         <v>0.4</v>
       </c>
       <c r="L8">
-        <v>0.29</v>
+        <v>0.28999999999999998</v>
       </c>
       <c r="M8">
         <v>0.05</v>
@@ -2147,7 +2207,7 @@
         <v>0.39</v>
       </c>
     </row>
-    <row r="9" spans="1:15">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>11</v>
       </c>
@@ -2158,13 +2218,13 @@
         <v>0.54</v>
       </c>
       <c r="D9">
-        <v>0.5600000000000001</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="E9">
         <v>0.51</v>
       </c>
       <c r="F9">
-        <v>0.5600000000000001</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="G9">
         <v>0.52</v>
@@ -2194,7 +2254,7 @@
         <v>0.34</v>
       </c>
     </row>
-    <row r="10" spans="1:15">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>12</v>
       </c>
@@ -2241,7 +2301,7 @@
         <v>0.16</v>
       </c>
     </row>
-    <row r="11" spans="1:15">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>13</v>
       </c>
@@ -2249,16 +2309,16 @@
         <v>0.53</v>
       </c>
       <c r="C11">
-        <v>0.58</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="D11">
-        <v>0.5600000000000001</v>
+        <v>0.56000000000000005</v>
       </c>
       <c r="E11">
         <v>0.62</v>
       </c>
       <c r="F11">
-        <v>0.58</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="G11">
         <v>0.64</v>
@@ -2288,7 +2348,7 @@
         <v>0.5</v>
       </c>
     </row>
-    <row r="12" spans="1:15">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>14</v>
       </c>
@@ -2311,7 +2371,7 @@
         <v>-0.03</v>
       </c>
       <c r="H12">
-        <v>0.29</v>
+        <v>0.28999999999999998</v>
       </c>
       <c r="I12">
         <v>0.03</v>
@@ -2332,10 +2392,10 @@
         <v>-0.08</v>
       </c>
       <c r="O12">
-        <v>-0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>15</v>
       </c>
@@ -2349,7 +2409,7 @@
         <v>-0.02</v>
       </c>
       <c r="E13">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="F13">
         <v>-0.04</v>
@@ -2382,7 +2442,7 @@
         <v>-0.05</v>
       </c>
     </row>
-    <row r="14" spans="1:15">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>16</v>
       </c>
@@ -2390,7 +2450,7 @@
         <v>0.12</v>
       </c>
       <c r="C14">
-        <v>0.14</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="D14">
         <v>0.16</v>
@@ -2429,7 +2489,7 @@
         <v>0.16</v>
       </c>
     </row>
-    <row r="15" spans="1:15">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>17</v>
       </c>
@@ -2464,7 +2524,7 @@
         <v>0.5</v>
       </c>
       <c r="L15">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="M15">
         <v>-0.05</v>
@@ -2482,11 +2542,11 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:O15"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>3</v>
       </c>
@@ -2533,7 +2593,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:15">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>4</v>
       </c>
@@ -2556,7 +2616,7 @@
         <v>0</v>
       </c>
       <c r="H2">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I2">
         <v>0</v>
@@ -2568,19 +2628,19 @@
         <v>0</v>
       </c>
       <c r="L2">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="M2">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="N2">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="O2">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>5</v>
       </c>
@@ -2615,19 +2675,19 @@
         <v>0</v>
       </c>
       <c r="L3">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="M3">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="N3">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="O3">
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>6</v>
       </c>
@@ -2662,19 +2722,19 @@
         <v>0</v>
       </c>
       <c r="L4">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="M4">
         <v>0</v>
       </c>
       <c r="N4">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="O4">
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>7</v>
       </c>
@@ -2703,13 +2763,13 @@
         <v>0</v>
       </c>
       <c r="J5">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="K5">
         <v>0</v>
       </c>
       <c r="L5">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="M5">
         <v>0</v>
@@ -2721,7 +2781,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:15">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>8</v>
       </c>
@@ -2756,19 +2816,19 @@
         <v>0</v>
       </c>
       <c r="L6">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="M6">
         <v>0</v>
       </c>
       <c r="N6">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="O6">
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:15">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>9</v>
       </c>
@@ -2797,30 +2857,30 @@
         <v>0</v>
       </c>
       <c r="J7">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="K7">
         <v>0</v>
       </c>
       <c r="L7">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="M7">
         <v>0</v>
       </c>
       <c r="N7">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="O7">
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B8">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="C8">
         <v>0</v>
@@ -2850,10 +2910,10 @@
         <v>0</v>
       </c>
       <c r="L8">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="M8">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="N8">
         <v>0</v>
@@ -2862,7 +2922,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:15">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>11</v>
       </c>
@@ -2897,10 +2957,10 @@
         <v>0</v>
       </c>
       <c r="L9">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="M9">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="N9">
         <v>0</v>
@@ -2909,7 +2969,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:15">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>12</v>
       </c>
@@ -2923,13 +2983,13 @@
         <v>0</v>
       </c>
       <c r="E10">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="F10">
         <v>0</v>
       </c>
       <c r="G10">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="H10">
         <v>0</v>
@@ -2941,22 +3001,22 @@
         <v>0</v>
       </c>
       <c r="K10">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="L10">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="M10">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="N10">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="O10">
-        <v>-0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>13</v>
       </c>
@@ -2985,57 +3045,57 @@
         <v>0</v>
       </c>
       <c r="J11">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="K11">
         <v>0</v>
       </c>
       <c r="L11">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="M11">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="N11">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="O11">
-        <v>-0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B12">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="C12">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="D12">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="E12">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="F12">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G12">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="H12">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I12">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="J12">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="K12">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="L12">
         <v>0</v>
@@ -3044,21 +3104,21 @@
         <v>0</v>
       </c>
       <c r="N12">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="O12">
-        <v>-0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:15">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B13">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="C13">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="D13">
         <v>0</v>
@@ -3073,16 +3133,16 @@
         <v>0</v>
       </c>
       <c r="H13">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="I13">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="J13">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="K13">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="L13">
         <v>0</v>
@@ -3097,27 +3157,27 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:15">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B14">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="C14">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="D14">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="E14">
         <v>0</v>
       </c>
       <c r="F14">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="G14">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="H14">
         <v>0</v>
@@ -3126,13 +3186,13 @@
         <v>0</v>
       </c>
       <c r="J14">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="K14">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="L14">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="M14">
         <v>0</v>
@@ -3144,7 +3204,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:15">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>17</v>
       </c>
@@ -3173,13 +3233,13 @@
         <v>0</v>
       </c>
       <c r="J15">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="K15">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="L15">
-        <v>-0</v>
+        <v>0</v>
       </c>
       <c r="M15">
         <v>0</v>
@@ -3197,11 +3257,11 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:Y37"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.2">
       <c r="B1" s="1" t="s">
         <v>18</v>
       </c>
@@ -3275,7 +3335,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="2" spans="1:25">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A2" s="1">
         <v>0</v>
       </c>
@@ -3349,7 +3409,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="3" spans="1:25">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -3405,7 +3465,7 @@
         <v>0.04</v>
       </c>
     </row>
-    <row r="4" spans="1:25">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -3416,7 +3476,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="5" spans="1:25">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A5" s="1">
         <v>3</v>
       </c>
@@ -3448,7 +3508,7 @@
         <v>0.15</v>
       </c>
       <c r="K5">
-        <v>0.14</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="L5">
         <v>0.13</v>
@@ -3469,7 +3529,7 @@
         <v>0.08</v>
       </c>
       <c r="R5">
-        <v>0.07000000000000001</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="S5">
         <v>0.06</v>
@@ -3490,7 +3550,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="6" spans="1:25">
+    <row r="6" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A6" s="1">
         <v>4</v>
       </c>
@@ -3522,7 +3582,7 @@
         <v>0.15</v>
       </c>
       <c r="K6">
-        <v>0.14</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="L6">
         <v>0.13</v>
@@ -3543,7 +3603,7 @@
         <v>0.08</v>
       </c>
       <c r="R6">
-        <v>0.07000000000000001</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="S6">
         <v>0.06</v>
@@ -3564,7 +3624,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="7" spans="1:25">
+    <row r="7" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A7" s="1">
         <v>5</v>
       </c>
@@ -3596,7 +3656,7 @@
         <v>0.15</v>
       </c>
       <c r="K7">
-        <v>0.14</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="L7">
         <v>0.13</v>
@@ -3617,7 +3677,7 @@
         <v>0.08</v>
       </c>
       <c r="R7">
-        <v>0.07000000000000001</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="S7">
         <v>0.06</v>
@@ -3638,7 +3698,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="8" spans="1:25">
+    <row r="8" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A8" s="1">
         <v>6</v>
       </c>
@@ -3670,7 +3730,7 @@
         <v>0.15</v>
       </c>
       <c r="K8">
-        <v>0.14</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="L8">
         <v>0.13</v>
@@ -3691,7 +3751,7 @@
         <v>0.08</v>
       </c>
       <c r="R8">
-        <v>0.07000000000000001</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="S8">
         <v>0.06</v>
@@ -3712,7 +3772,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="9" spans="1:25">
+    <row r="9" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A9" s="1">
         <v>7</v>
       </c>
@@ -3786,7 +3846,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="10" spans="1:25">
+    <row r="10" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A10" s="1">
         <v>8</v>
       </c>
@@ -3860,7 +3920,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="11" spans="1:25">
+    <row r="11" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A11" s="1">
         <v>9</v>
       </c>
@@ -3934,7 +3994,7 @@
         <v>134</v>
       </c>
     </row>
-    <row r="12" spans="1:25">
+    <row r="12" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A12" s="1">
         <v>10</v>
       </c>
@@ -4008,7 +4068,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="13" spans="1:25">
+    <row r="13" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A13" s="1">
         <v>11</v>
       </c>
@@ -4025,7 +4085,7 @@
         <v>0.63</v>
       </c>
       <c r="M13">
-        <v>0.58</v>
+        <v>0.57999999999999996</v>
       </c>
       <c r="N13">
         <v>0.53</v>
@@ -4043,7 +4103,7 @@
         <v>0.33</v>
       </c>
       <c r="S13">
-        <v>0.28</v>
+        <v>0.28000000000000003</v>
       </c>
       <c r="T13">
         <v>0.23</v>
@@ -4058,12 +4118,12 @@
         <v>0.96</v>
       </c>
     </row>
-    <row r="14" spans="1:25">
+    <row r="14" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A14" s="1">
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:25">
+    <row r="15" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A15" s="1">
         <v>13</v>
       </c>
@@ -4107,7 +4167,7 @@
         <v>0.06</v>
       </c>
       <c r="O15">
-        <v>0.07000000000000001</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="P15">
         <v>0.08</v>
@@ -4137,7 +4197,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="16" spans="1:25">
+    <row r="16" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A16" s="1">
         <v>14</v>
       </c>
@@ -4181,7 +4241,7 @@
         <v>0.06</v>
       </c>
       <c r="O16">
-        <v>0.07000000000000001</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="P16">
         <v>0.08</v>
@@ -4211,7 +4271,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="17" spans="1:24">
+    <row r="17" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A17" s="1">
         <v>15</v>
       </c>
@@ -4285,7 +4345,7 @@
         <v>138</v>
       </c>
     </row>
-    <row r="18" spans="1:24">
+    <row r="18" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A18" s="1">
         <v>16</v>
       </c>
@@ -4344,7 +4404,7 @@
         <v>0.05</v>
       </c>
       <c r="V18">
-        <v>0.07000000000000001</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="W18">
         <v>0</v>
@@ -4353,7 +4413,7 @@
         <v>139</v>
       </c>
     </row>
-    <row r="19" spans="1:24">
+    <row r="19" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A19" s="1">
         <v>17</v>
       </c>
@@ -4412,7 +4472,7 @@
         <v>0.05</v>
       </c>
       <c r="V19">
-        <v>0.07000000000000001</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="W19">
         <v>0</v>
@@ -4421,7 +4481,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="20" spans="1:24">
+    <row r="20" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A20" s="1">
         <v>18</v>
       </c>
@@ -4489,7 +4549,7 @@
         <v>141</v>
       </c>
     </row>
-    <row r="21" spans="1:24">
+    <row r="21" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A21" s="1">
         <v>19</v>
       </c>
@@ -4533,18 +4593,18 @@
         <v>0.38</v>
       </c>
       <c r="V21">
-        <v>0.57</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="W21">
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:24">
+    <row r="22" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A22" s="1">
         <v>20</v>
       </c>
     </row>
-    <row r="23" spans="1:24">
+    <row r="23" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A23" s="1">
         <v>21</v>
       </c>
@@ -4612,7 +4672,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="24" spans="1:24">
+    <row r="24" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A24" s="1">
         <v>22</v>
       </c>
@@ -4680,7 +4740,7 @@
         <v>143</v>
       </c>
     </row>
-    <row r="25" spans="1:24">
+    <row r="25" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A25" s="1">
         <v>23</v>
       </c>
@@ -4748,7 +4808,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="26" spans="1:24">
+    <row r="26" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A26" s="1">
         <v>24</v>
       </c>
@@ -4816,7 +4876,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="27" spans="1:24">
+    <row r="27" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A27" s="1">
         <v>25</v>
       </c>
@@ -4875,7 +4935,7 @@
         <v>0.05</v>
       </c>
       <c r="V27">
-        <v>0.07000000000000001</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="W27">
         <v>0</v>
@@ -4884,7 +4944,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="28" spans="1:24">
+    <row r="28" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A28" s="1">
         <v>26</v>
       </c>
@@ -4892,7 +4952,7 @@
         <v>0.06</v>
       </c>
       <c r="J28">
-        <v>0.07000000000000001</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="K28">
         <v>0.08</v>
@@ -4934,12 +4994,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:24">
+    <row r="29" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A29" s="1">
         <v>27</v>
       </c>
     </row>
-    <row r="30" spans="1:24">
+    <row r="30" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A30" s="1">
         <v>28</v>
       </c>
@@ -5007,7 +5067,7 @@
         <v>147</v>
       </c>
     </row>
-    <row r="31" spans="1:24">
+    <row r="31" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A31" s="1">
         <v>29</v>
       </c>
@@ -5075,7 +5135,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="32" spans="1:24">
+    <row r="32" spans="1:24" x14ac:dyDescent="0.2">
       <c r="A32" s="1">
         <v>30</v>
       </c>
@@ -5143,7 +5203,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="33" spans="1:25">
+    <row r="33" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A33" s="1">
         <v>31</v>
       </c>
@@ -5211,7 +5271,7 @@
         <v>150</v>
       </c>
     </row>
-    <row r="34" spans="1:25">
+    <row r="34" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A34" s="1">
         <v>32</v>
       </c>
@@ -5279,7 +5339,7 @@
         <v>151</v>
       </c>
     </row>
-    <row r="35" spans="1:25">
+    <row r="35" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A35" s="1">
         <v>33</v>
       </c>
@@ -5329,12 +5389,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:25">
+    <row r="36" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A36" s="1">
         <v>34</v>
       </c>
     </row>
-    <row r="37" spans="1:25">
+    <row r="37" spans="1:25" x14ac:dyDescent="0.2">
       <c r="A37" s="1">
         <v>35</v>
       </c>
@@ -5396,11 +5456,11 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
   <dimension ref="A1:O15"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:15">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.2">
       <c r="B1" s="1" t="s">
         <v>25</v>
       </c>
@@ -5444,7 +5504,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="2" spans="1:15">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>112</v>
       </c>
@@ -5467,7 +5527,7 @@
         <v>0.06</v>
       </c>
       <c r="H2">
-        <v>0.07000000000000001</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="I2">
         <v>0.08</v>
@@ -5491,7 +5551,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="3" spans="1:15">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>113</v>
       </c>
@@ -5505,7 +5565,7 @@
         <v>0.06</v>
       </c>
       <c r="E3">
-        <v>0.07000000000000001</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="F3">
         <v>0.08</v>
@@ -5532,13 +5592,13 @@
         <v>0.13</v>
       </c>
       <c r="N3">
-        <v>0.14</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="O3" t="s">
         <v>123</v>
       </c>
     </row>
-    <row r="4" spans="1:15">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>114</v>
       </c>
@@ -5585,7 +5645,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="5" spans="1:15">
+    <row r="5" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>115</v>
       </c>
@@ -5632,7 +5692,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="6" spans="1:15">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>116</v>
       </c>
@@ -5679,7 +5739,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="7" spans="1:15">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>117</v>
       </c>
@@ -5726,7 +5786,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="8" spans="1:15">
+    <row r="8" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>118</v>
       </c>
@@ -5752,7 +5812,7 @@
         <v>0.13</v>
       </c>
       <c r="I8">
-        <v>0.14</v>
+        <v>0.14000000000000001</v>
       </c>
       <c r="J8">
         <v>0.16</v>
@@ -5773,7 +5833,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="9" spans="1:15">
+    <row r="9" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>119</v>
       </c>
@@ -5805,7 +5865,7 @@
         <v>0.06</v>
       </c>
       <c r="K9">
-        <v>0.07000000000000001</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="L9">
         <v>0.09</v>
@@ -5820,7 +5880,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="10" spans="1:15">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>120</v>
       </c>
@@ -5834,7 +5894,7 @@
         <v>0.61</v>
       </c>
       <c r="E10">
-        <v>0.57</v>
+        <v>0.56999999999999995</v>
       </c>
       <c r="F10">
         <v>0.52</v>
@@ -5867,7 +5927,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="11" spans="1:15">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>121</v>
       </c>
@@ -5914,12 +5974,12 @@
         <v>124</v>
       </c>
     </row>
-    <row r="12" spans="1:15">
+    <row r="12" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>122</v>
       </c>
       <c r="B12">
-        <v>0.07000000000000001</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="C12">
         <v>0.06</v>
@@ -5961,7 +6021,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="13" spans="1:15">
+    <row r="13" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>15</v>
       </c>
@@ -6008,7 +6068,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="14" spans="1:15">
+    <row r="14" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>17</v>
       </c>
@@ -6055,7 +6115,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="15" spans="1:15">
+    <row r="15" spans="1:15" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>16</v>
       </c>
@@ -6075,28 +6135,28 @@
         <v>0.06</v>
       </c>
       <c r="G15">
-        <v>0.07000000000000001</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="H15">
-        <v>0.07000000000000001</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="I15">
-        <v>0.07000000000000001</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="J15">
-        <v>0.07000000000000001</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="K15">
-        <v>0.07000000000000001</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="L15">
-        <v>0.07000000000000001</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="M15">
-        <v>0.07000000000000001</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="N15">
-        <v>0.07000000000000001</v>
+        <v>7.0000000000000007E-2</v>
       </c>
       <c r="O15" t="s">
         <v>123</v>
@@ -6108,11 +6168,11 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:N3"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A1" s="1" t="s">
         <v>22</v>
       </c>
@@ -6156,7 +6216,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="2" spans="1:14">
+    <row r="2" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>124</v>
       </c>
@@ -6176,7 +6236,7 @@
         <v>0.6</v>
       </c>
       <c r="G2">
-        <v>0.55</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="H2">
         <v>0.5</v>
@@ -6200,7 +6260,7 @@
         <v>0.2</v>
       </c>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3" spans="1:14" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>123</v>
       </c>
@@ -6226,7 +6286,7 @@
         <v>0.5</v>
       </c>
       <c r="I3">
-        <v>0.55</v>
+        <v>0.55000000000000004</v>
       </c>
       <c r="J3">
         <v>0.6</v>

</xml_diff>